<commit_message>
fix(data): guard representative counter charge exhaustion
</commit_message>
<xml_diff>
--- a/config/data/ConditionExpression.xlsx
+++ b/config/data/ConditionExpression.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ConditionExpression" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ConditionExpression" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -691,19 +691,17 @@
       </c>
     </row>
     <row r="9">
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>24201</t>
-        </is>
+      <c r="B9" t="n">
+        <v>24201</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>probe.clara.condition.true</t>
+          <t>program.clara.condition.has-counter-charge</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>{"type":"Constant","value":true}</t>
+          <t>{"type":"Compare","left_expression_id":24204,"comparison":"Greater","right_expression_id":24202}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(divergent-universe): verify footstep lifecycle consumers
Retain production bindings in transformation, linked-actor and unitless-countdown probes. Guard representative Clara counter admission with a present live owner without consuming unavailable-owner charges. Preserve the explicit internal-counter binding gap and project-policy accuracy boundary.

Author the bounded guard through clean openpyxl workbooks and regenerate Sora output. Rebind configuration-sensitive public routes and the shared current-state manifest without removing semantic assertions.

Verified formatting, affected-package Clippy and full tests, remaining workspace tests, production generation drift, workbook preservation, source policy, native-handler audit, documentation links and exact-once dispositions.
</commit_message>
<xml_diff>
--- a/config/data/ConditionExpression.xlsx
+++ b/config/data/ConditionExpression.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J64"/>
+  <dimension ref="A1:J66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12.7109375" customWidth="1" min="1" max="1"/>
@@ -696,12 +696,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>program.clara.condition.has-counter-charge</t>
+          <t>program.clara.condition.admitted-counter-owner</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>{"type":"Compare","left_expression_id":24204,"comparison":"Greater","right_expression_id":24202}</t>
+          <t>{"type":"All","condition_ids":[24202,24203]}</t>
         </is>
       </c>
     </row>
@@ -1621,6 +1621,36 @@
       <c r="D64" t="inlineStr">
         <is>
           <t>{"type":"SelectorCardinality","selector_id":1030411,"minimum_count":1,"maximum_count":2}</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" t="n">
+        <v>24202</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>program.clara.condition.has-counter-charge</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>{"type":"Compare","left_expression_id":24204,"comparison":"Greater","right_expression_id":24202}</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" t="n">
+        <v>24203</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>program.clara.condition.has-present-owner</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>{"type":"SelectorCardinality","selector_id":24251,"minimum_count":1,"maximum_count":1}</t>
         </is>
       </c>
     </row>

</xml_diff>